<commit_message>
feat(phase-b): add second secondary persona
</commit_message>
<xml_diff>
--- a/phase-b/phase-b-personas-and-cast.xlsx
+++ b/phase-b/phase-b-personas-and-cast.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="1" r:id="Rfb46623dfe9b4e4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cast" sheetId="2" r:id="R4c81b6ef485e4f61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence map" sheetId="3" r:id="R2e0bc90fbe634174"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario #1" sheetId="4" r:id="R88381cf286774e2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario #2" sheetId="5" r:id="R4b2792b2efb5403b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario #3" sheetId="6" r:id="R001fd33a6b84445a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="1" r:id="Rb9dc9098233a4371"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cast" sheetId="2" r:id="R62c6d0de86db4895"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence map" sheetId="3" r:id="R82adbb1f644247f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario #1" sheetId="4" r:id="R231400425f4f45ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario #2" sheetId="5" r:id="Ra0a0a8b59c014a4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario #3" sheetId="6" r:id="R8f684165dc774d70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario #4" sheetId="7" r:id="R619b238ad69f4e72"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,7 +19,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="12">
+  <x:fonts count="19">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -86,8 +87,49 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF8A5A00"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF8A5A00"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FF243B53"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF243B53"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF667085"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="13">
+  <x:fills count="28">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -147,6 +189,81 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF6F9FC7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF0CF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD5E1E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8E0C8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2E5C84"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF243B53"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9E7F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF0CF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD5E1E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8E0C8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2E5C84"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFA6C5D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF243B53"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9E7F4"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -338,7 +455,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="133">
+  <x:cellXfs count="171">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -734,6 +851,98 @@
     <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="20" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="20" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="21" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="22" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="23" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="23" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -788,10 +997,7 @@
             <c:v>Pina</c:v>
           </c:tx>
           <c:spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="C58A36"/>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="23813">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
               <a:solidFill>
                 <a:srgbClr val="C58A36"/>
               </a:solidFill>
@@ -823,10 +1029,7 @@
             <c:v>Elena</c:v>
           </c:tx>
           <c:spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="2F6FB2"/>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="23813">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
               <a:solidFill>
                 <a:srgbClr val="2F6FB2"/>
               </a:solidFill>
@@ -855,17 +1058,14 @@
           <c:idx val="2"/>
           <c:order val="2"/>
           <c:tx>
-            <c:v>Renato</c:v>
+            <c:v>Amina</c:v>
           </c:tx>
           <c:spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="4C8C8A"/>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="23813">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
               <a:solidFill>
-                <a:srgbClr val="4C8C8A"/>
+                <a:srgbClr val="8A4F7D"/>
               </a:solidFill>
-              <a:prstDash val="solid"/>
+              <a:prstDash val="dashDot"/>
             </a:ln>
           </c:spPr>
           <c:cat>
@@ -879,6 +1079,38 @@
           <c:val>
             <c:numRef>
               <c:f>'Cast'!$D$44:$D$49</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:v>Renato</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="4C8C8A"/>
+              </a:solidFill>
+              <a:prstDash val="dot"/>
+            </a:ln>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Cast'!$A$44:$A$49</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Cast'!$E$44:$E$49</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="0"/>
@@ -944,7 +1176,7 @@
         <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr>
+            <a:defRPr sz="750">
               <a:latin typeface="Arial"/>
               <a:ea typeface="Arial"/>
               <a:cs typeface="Arial"/>
@@ -1380,6 +1612,145 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/drawings/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:r>
+              <a:rPr sz="975">
+                <a:latin typeface="Arial"/>
+                <a:ea typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:rPr>
+              <a:t>Profilo C&amp;A - Amina</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr sz="975">
+              <a:latin typeface="Arial"/>
+              <a:ea typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:plotArea>
+      <c:radarChart>
+        <c:radarStyle val="standard"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Punteggio</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="8A4F7D"/>
+              </a:solidFill>
+              <a:prstDash val="dashDot"/>
+            </a:ln>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Scenario #4'!$J$25:$J$30</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Scenario #4'!$K$25:$K$30</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
+      </c:radarChart>
+      <c:catAx>
+        <c:axId val="48650112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="48672768"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="48672768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:crossAx val="48650112"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
@@ -1392,7 +1763,7 @@
     <xdr:to>
       <xdr:col>12</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>39</xdr:row>
+      <xdr:row>40</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1406,7 +1777,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb4cf4d58508848f6"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R40c4fdaff3e64c2d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1441,7 +1812,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R48a1aa4196c540dd"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R084733f41045491e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1476,7 +1847,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R39725270f16b4558"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R26cfc401e78b43a2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1511,7 +1882,42 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R55ef52bc94b34ca3"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1d357e1fec254fc2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="1" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rca0b1e57448d446a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1837,7 +2243,7 @@
         <x:v>Gerarchia</x:v>
       </x:c>
       <x:c r="B6" s="16" t="str">
-        <x:v>Pina = protagonista; Elena = personaggio secondario; Renato = personaggio aggiuntivo.</x:v>
+        <x:v>Pina = protagonista; Elena e Amina = personaggi secondari; Renato = personaggio aggiuntivo.</x:v>
       </x:c>
       <x:c r="C6" s="2"/>
       <x:c r="D6" s="2"/>
@@ -1943,8 +2349,12 @@
       <x:c r="P10" s="2"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="2"/>
-      <x:c r="B11" s="2"/>
+      <x:c r="A11" s="2" t="str">
+        <x:v>Equità del cast</x:v>
+      </x:c>
+      <x:c r="B11" s="2" t="str">
+        <x:v>La varietà di genere, origine, lingua e struttura familiare è inclusa quando modifica scenari e requisiti, non come tratto decorativo.</x:v>
+      </x:c>
       <x:c r="C11" s="2"/>
       <x:c r="D11" s="2"/>
       <x:c r="E11" s="2"/>
@@ -3137,21 +3547,21 @@
     </x:row>
     <x:row r="9" ht="46" customHeight="1">
       <x:c r="A9" s="39" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B9" s="34" t="str">
-        <x:v>Renato Bellini</x:v>
+        <x:v>Amina Rahman</x:v>
       </x:c>
       <x:c r="C9" s="34" t="str">
-        <x:v>Personaggio aggiuntivo</x:v>
+        <x:v>Personaggio secondario</x:v>
       </x:c>
       <x:c r="D9" s="34" t="str">
-        <x:v>Utente diretto, 65-74 anni, autonomia digitale moderata</x:v>
+        <x:v>Caregiver convivente, 40-55 anni, competenza digitale media</x:v>
       </x:c>
       <x:c r="E9" s="34" t="str">
-        <x:v>Il controllo oculistico senza chiamare il figlio</x:v>
-      </x:c>
-      <x:c r="F9" s="48" t="str">
+        <x:v>La fisioterapia prima del turno</x:v>
+      </x:c>
+      <x:c r="F9" s="155" t="str">
         <x:v>Da validare</x:v>
       </x:c>
       <x:c r="G9" s="35" t="n">
@@ -3161,16 +3571,16 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="I9" s="35" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J9" s="35" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="J9" s="35" t="n">
-        <x:v>3</x:v>
-      </x:c>
       <x:c r="K9" s="35" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L9" s="36" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="M9" s="2"/>
       <x:c r="N9" s="2"/>
@@ -3178,18 +3588,42 @@
       <x:c r="P9" s="2"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="2"/>
-      <x:c r="B10" s="2"/>
-      <x:c r="C10" s="2"/>
-      <x:c r="D10" s="2"/>
-      <x:c r="E10" s="2"/>
-      <x:c r="F10" s="2"/>
-      <x:c r="G10" s="2"/>
-      <x:c r="H10" s="2"/>
-      <x:c r="I10" s="2"/>
-      <x:c r="J10" s="2"/>
-      <x:c r="K10" s="2"/>
-      <x:c r="L10" s="2"/>
+      <x:c r="A10" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B10" s="2" t="str">
+        <x:v>Renato Bellini</x:v>
+      </x:c>
+      <x:c r="C10" s="2" t="str">
+        <x:v>Personaggio aggiuntivo</x:v>
+      </x:c>
+      <x:c r="D10" s="2" t="str">
+        <x:v>Utente diretto, 65-74 anni, autonomia digitale moderata</x:v>
+      </x:c>
+      <x:c r="E10" s="2" t="str">
+        <x:v>Il controllo oculistico senza chiamare il figlio</x:v>
+      </x:c>
+      <x:c r="F10" s="154" t="str">
+        <x:v>Da validare</x:v>
+      </x:c>
+      <x:c r="G10" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H10" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I10" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J10" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K10" s="2" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L10" s="2" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="M10" s="2"/>
       <x:c r="N10" s="2"/>
       <x:c r="O10" s="2"/>
@@ -3372,25 +3806,25 @@
       <x:c r="D16" s="2" t="str"/>
       <x:c r="E16" s="2"/>
       <x:c r="F16" s="73" t="str">
-        <x:v>Renato</x:v>
-      </x:c>
-      <x:c r="G16" s="89" t="n">
+        <x:v>Amina</x:v>
+      </x:c>
+      <x:c r="G16" s="156" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="H16" s="89" t="n">
+      <x:c r="H16" s="156" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="I16" s="93" t="n">
+      <x:c r="I16" s="157" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J16" s="158" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="J16" s="89" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="K16" s="85" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="L16" s="85" t="n">
-        <x:v>4</x:v>
+      <x:c r="K16" s="159" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="L16" s="157" t="n">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="M16" s="2"/>
       <x:c r="N16" s="2"/>
@@ -3399,25 +3833,39 @@
     </x:row>
     <x:row r="17" ht="35" customHeight="1">
       <x:c r="A17" s="70" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B17" s="71" t="str">
+        <x:v>Amina</x:v>
+      </x:c>
+      <x:c r="C17" s="71" t="str">
+        <x:v>Secondaria</x:v>
+      </x:c>
+      <x:c r="D17" s="72" t="str">
+        <x:v>Caregiver convivente: mediazione linguistica, coordinamento familiare e uso interrotto.</x:v>
+      </x:c>
+      <x:c r="E17" s="2"/>
+      <x:c r="F17" s="2" t="str">
+        <x:v>Renato</x:v>
+      </x:c>
+      <x:c r="G17" s="160" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B17" s="71" t="str">
-        <x:v>Renato</x:v>
-      </x:c>
-      <x:c r="C17" s="71" t="str">
-        <x:v>Aggiuntivo</x:v>
-      </x:c>
-      <x:c r="D17" s="72" t="str">
-        <x:v>Controlla efficienza, tono non paternalistico e accessibilità per utenti più autonomi.</x:v>
-      </x:c>
-      <x:c r="E17" s="2"/>
-      <x:c r="F17" s="2"/>
-      <x:c r="G17" s="2"/>
-      <x:c r="H17" s="2"/>
-      <x:c r="I17" s="2"/>
-      <x:c r="J17" s="2"/>
-      <x:c r="K17" s="2"/>
-      <x:c r="L17" s="2"/>
+      <x:c r="H17" s="160" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I17" s="161" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J17" s="160" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K17" s="162" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L17" s="162" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="M17" s="2"/>
       <x:c r="N17" s="2"/>
       <x:c r="O17" s="2"/>
@@ -3456,10 +3904,18 @@
       <x:c r="P18" s="2"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="2"/>
-      <x:c r="B19" s="2"/>
-      <x:c r="C19" s="2"/>
-      <x:c r="D19" s="2"/>
+      <x:c r="A19" s="2" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B19" s="2" t="str">
+        <x:v>Renato</x:v>
+      </x:c>
+      <x:c r="C19" s="2" t="str">
+        <x:v>Aggiuntivo</x:v>
+      </x:c>
+      <x:c r="D19" s="2" t="str">
+        <x:v>Controlla efficienza, tono non paternalistico e accessibilità per utenti più autonomi.</x:v>
+      </x:c>
       <x:c r="E19" s="2"/>
       <x:c r="F19" s="2"/>
       <x:c r="G19" s="2"/>
@@ -3920,19 +4376,21 @@
       <x:c r="P42" s="2"/>
     </x:row>
     <x:row r="43" ht="30" customHeight="1">
-      <x:c r="A43" s="22" t="str">
+      <x:c r="A43" s="163" t="str">
         <x:v>Dimensione</x:v>
       </x:c>
-      <x:c r="B43" s="22" t="str">
+      <x:c r="B43" s="163" t="str">
         <x:v>Pina</x:v>
       </x:c>
-      <x:c r="C43" s="22" t="str">
+      <x:c r="C43" s="163" t="str">
         <x:v>Elena</x:v>
       </x:c>
-      <x:c r="D43" s="22" t="str">
+      <x:c r="D43" s="163" t="str">
+        <x:v>Amina</x:v>
+      </x:c>
+      <x:c r="E43" s="164" t="str">
         <x:v>Renato</x:v>
       </x:c>
-      <x:c r="E43" s="2"/>
       <x:c r="F43" s="2"/>
       <x:c r="G43" s="2"/>
       <x:c r="H43" s="2"/>
@@ -3958,7 +4416,9 @@
       <x:c r="D44" s="28" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="E44" s="2"/>
+      <x:c r="E44" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="F44" s="2"/>
       <x:c r="G44" s="2"/>
       <x:c r="H44" s="2"/>
@@ -3984,7 +4444,9 @@
       <x:c r="D45" s="32" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="E45" s="2"/>
+      <x:c r="E45" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="F45" s="2"/>
       <x:c r="G45" s="2"/>
       <x:c r="H45" s="2"/>
@@ -4008,9 +4470,11 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="D46" s="32" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E46" s="2" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="E46" s="2"/>
       <x:c r="F46" s="2"/>
       <x:c r="G46" s="2"/>
       <x:c r="H46" s="2"/>
@@ -4034,9 +4498,11 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="D47" s="32" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E47" s="2" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="E47" s="2"/>
       <x:c r="F47" s="2"/>
       <x:c r="G47" s="2"/>
       <x:c r="H47" s="2"/>
@@ -4060,9 +4526,11 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="D48" s="32" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E48" s="2" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="E48" s="2"/>
       <x:c r="F48" s="2"/>
       <x:c r="G48" s="2"/>
       <x:c r="H48" s="2"/>
@@ -4086,9 +4554,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="D49" s="36" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E49" s="2" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="E49" s="2"/>
       <x:c r="F49" s="2"/>
       <x:c r="G49" s="2"/>
       <x:c r="H49" s="2"/>
@@ -4310,7 +4780,7 @@
     <x:mergeCell ref="A42:D42"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ace7c09e7bd4431"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2eda4a0203e44c36"/>
 </x:worksheet>
 </file>
 
@@ -4833,13 +5303,27 @@
       <x:c r="P17" s="2"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="2"/>
-      <x:c r="B18" s="2"/>
-      <x:c r="C18" s="2"/>
-      <x:c r="D18" s="2"/>
-      <x:c r="E18" s="2"/>
-      <x:c r="F18" s="2"/>
-      <x:c r="G18" s="2"/>
+      <x:c r="A18" s="2" t="str">
+        <x:v>Amina</x:v>
+      </x:c>
+      <x:c r="B18" s="2" t="str">
+        <x:v>Gestione convivente e interruzioni</x:v>
+      </x:c>
+      <x:c r="C18" s="2" t="str">
+        <x:v>Segmento B - Q1-Q2, Q6</x:v>
+      </x:c>
+      <x:c r="D18" s="2" t="str">
+        <x:v>Ipotesi narrativa e contesto d'uso</x:v>
+      </x:c>
+      <x:c r="E18" s="165" t="str">
+        <x:v>Da validare</x:v>
+      </x:c>
+      <x:c r="F18" s="2" t="str">
+        <x:v>Ricostruire un episodio reale e i tempi</x:v>
+      </x:c>
+      <x:c r="G18" s="2" t="str">
+        <x:v>Non attribuire il carico alla sola origine migratoria</x:v>
+      </x:c>
       <x:c r="H18" s="2"/>
       <x:c r="I18" s="2"/>
       <x:c r="J18" s="2"/>
@@ -4851,13 +5335,27 @@
       <x:c r="P18" s="2"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="2"/>
-      <x:c r="B19" s="2"/>
-      <x:c r="C19" s="2"/>
-      <x:c r="D19" s="2"/>
-      <x:c r="E19" s="2"/>
-      <x:c r="F19" s="2"/>
-      <x:c r="G19" s="2"/>
+      <x:c r="A19" s="2" t="str">
+        <x:v>Amina</x:v>
+      </x:c>
+      <x:c r="B19" s="2" t="str">
+        <x:v>Delega, identità e coordinamento</x:v>
+      </x:c>
+      <x:c r="C19" s="2" t="str">
+        <x:v>Segmento B - Q3-Q4</x:v>
+      </x:c>
+      <x:c r="D19" s="2" t="str">
+        <x:v>Obiettivo HPHP e scenario</x:v>
+      </x:c>
+      <x:c r="E19" s="165" t="str">
+        <x:v>Da validare</x:v>
+      </x:c>
+      <x:c r="F19" s="2" t="str">
+        <x:v>Verificare ruoli, permessi e duplicazioni</x:v>
+      </x:c>
+      <x:c r="G19" s="2" t="str">
+        <x:v>Distinguere convivenza da delega legale</x:v>
+      </x:c>
       <x:c r="H19" s="2"/>
       <x:c r="I19" s="2"/>
       <x:c r="J19" s="2"/>
@@ -4869,13 +5367,27 @@
       <x:c r="P19" s="2"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="2"/>
-      <x:c r="B20" s="2"/>
-      <x:c r="C20" s="2"/>
-      <x:c r="D20" s="2"/>
-      <x:c r="E20" s="2"/>
-      <x:c r="F20" s="2"/>
-      <x:c r="G20" s="2"/>
+      <x:c r="A20" s="2" t="str">
+        <x:v>Amina</x:v>
+      </x:c>
+      <x:c r="B20" s="2" t="str">
+        <x:v>Comprensione e condizioni di fiducia</x:v>
+      </x:c>
+      <x:c r="C20" s="2" t="str">
+        <x:v>Segmento B - Q4-Q5</x:v>
+      </x:c>
+      <x:c r="D20" s="2" t="str">
+        <x:v>Criticità linguistiche ipotizzate</x:v>
+      </x:c>
+      <x:c r="E20" s="165" t="str">
+        <x:v>Da validare</x:v>
+      </x:c>
+      <x:c r="F20" s="2" t="str">
+        <x:v>Osservare termini e strategie di chiarimento</x:v>
+      </x:c>
+      <x:c r="G20" s="2" t="str">
+        <x:v>Non confondere italiano L2 con bassa competenza digitale</x:v>
+      </x:c>
       <x:c r="H20" s="2"/>
       <x:c r="I20" s="2"/>
       <x:c r="J20" s="2"/>
@@ -6918,7 +7430,7 @@
     <x:mergeCell ref="E21:P21"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ea0af0528c3498d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1e06d1348d548d1"/>
 </x:worksheet>
 </file>
 
@@ -8226,7 +8738,7 @@
     <x:mergeCell ref="E21:P21"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33675b32915f46e8"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf9974b9f3a54863"/>
 </x:worksheet>
 </file>
 
@@ -9534,6 +10046,741 @@
     <x:mergeCell ref="E21:P21"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cd5fc3ff0974895"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra828350eeb6e430c"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="92" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="65" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="3" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="13" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="13" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="13" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="13" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="13" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="13" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="13" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="13" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1"/>
+      <x:c r="B1"/>
+      <x:c r="C1"/>
+      <x:c r="D1"/>
+      <x:c r="E1"/>
+      <x:c r="F1"/>
+      <x:c r="G1"/>
+      <x:c r="H1"/>
+      <x:c r="I1"/>
+      <x:c r="J1"/>
+      <x:c r="K1"/>
+      <x:c r="L1"/>
+      <x:c r="M1"/>
+      <x:c r="N1"/>
+      <x:c r="O1"/>
+      <x:c r="P1"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="142" t="str">
+        <x:v>Amina Rahman - Personaggio secondario</x:v>
+      </x:c>
+      <x:c r="B2"/>
+      <x:c r="C2"/>
+      <x:c r="D2"/>
+      <x:c r="E2"/>
+      <x:c r="F2"/>
+      <x:c r="G2"/>
+      <x:c r="H2"/>
+      <x:c r="I2"/>
+      <x:c r="J2"/>
+      <x:c r="K2"/>
+      <x:c r="L2"/>
+      <x:c r="M2"/>
+      <x:c r="N2"/>
+      <x:c r="O2"/>
+      <x:c r="P2"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3"/>
+      <x:c r="B3"/>
+      <x:c r="C3"/>
+      <x:c r="D3"/>
+      <x:c r="E3"/>
+      <x:c r="F3"/>
+      <x:c r="G3"/>
+      <x:c r="H3"/>
+      <x:c r="I3"/>
+      <x:c r="J3"/>
+      <x:c r="K3"/>
+      <x:c r="L3"/>
+      <x:c r="M3"/>
+      <x:c r="N3"/>
+      <x:c r="O3"/>
+      <x:c r="P3"/>
+    </x:row>
+    <x:row r="4" ht="30" customHeight="1">
+      <x:c r="A4" s="167" t="str">
+        <x:v>Scenario</x:v>
+      </x:c>
+      <x:c r="B4" s="152" t="str">
+        <x:v>La fisioterapia prima del turno</x:v>
+      </x:c>
+      <x:c r="C4"/>
+      <x:c r="D4"/>
+      <x:c r="E4"/>
+      <x:c r="F4"/>
+      <x:c r="G4"/>
+      <x:c r="H4"/>
+      <x:c r="I4"/>
+      <x:c r="J4"/>
+      <x:c r="K4"/>
+      <x:c r="L4"/>
+      <x:c r="M4"/>
+      <x:c r="N4"/>
+      <x:c r="O4"/>
+      <x:c r="P4"/>
+    </x:row>
+    <x:row r="5" ht="30" customHeight="1">
+      <x:c r="A5" s="167" t="str">
+        <x:v>Livello nel cast</x:v>
+      </x:c>
+      <x:c r="B5" s="152" t="str">
+        <x:v>Personaggio secondario</x:v>
+      </x:c>
+      <x:c r="C5"/>
+      <x:c r="D5"/>
+      <x:c r="E5"/>
+      <x:c r="F5"/>
+      <x:c r="G5"/>
+      <x:c r="H5"/>
+      <x:c r="I5"/>
+      <x:c r="J5"/>
+      <x:c r="K5"/>
+      <x:c r="L5"/>
+      <x:c r="M5"/>
+      <x:c r="N5"/>
+      <x:c r="O5"/>
+      <x:c r="P5"/>
+    </x:row>
+    <x:row r="6" ht="30" customHeight="1">
+      <x:c r="A6" s="167" t="str">
+        <x:v>Segmento</x:v>
+      </x:c>
+      <x:c r="B6" s="152" t="str">
+        <x:v>Caregiver convivente, 40-55 anni, competenza digitale media; italiana L2</x:v>
+      </x:c>
+      <x:c r="C6"/>
+      <x:c r="D6"/>
+      <x:c r="E6"/>
+      <x:c r="F6"/>
+      <x:c r="G6"/>
+      <x:c r="H6"/>
+      <x:c r="I6"/>
+      <x:c r="J6"/>
+      <x:c r="K6"/>
+      <x:c r="L6"/>
+      <x:c r="M6"/>
+      <x:c r="N6"/>
+      <x:c r="O6"/>
+      <x:c r="P6"/>
+    </x:row>
+    <x:row r="7" ht="30" customHeight="1">
+      <x:c r="A7" s="167" t="str">
+        <x:v>Stato dell'evidenza</x:v>
+      </x:c>
+      <x:c r="B7" s="152" t="str">
+        <x:v>Ipotesi narrativa da validare con interviste del Segmento B</x:v>
+      </x:c>
+      <x:c r="C7"/>
+      <x:c r="D7"/>
+      <x:c r="E7"/>
+      <x:c r="F7"/>
+      <x:c r="G7"/>
+      <x:c r="H7"/>
+      <x:c r="I7"/>
+      <x:c r="J7"/>
+      <x:c r="K7"/>
+      <x:c r="L7"/>
+      <x:c r="M7"/>
+      <x:c r="N7"/>
+      <x:c r="O7"/>
+      <x:c r="P7"/>
+    </x:row>
+    <x:row r="8" ht="30" customHeight="1">
+      <x:c r="A8" s="167" t="str">
+        <x:v>Citazione provvisoria</x:v>
+      </x:c>
+      <x:c r="B8" s="152" t="str">
+        <x:v>Le cose di casa le organizzo io; con certe parole dell'ospedale, però, devo prima capire bene che cosa stanno chiedendo.</x:v>
+      </x:c>
+      <x:c r="C8"/>
+      <x:c r="D8"/>
+      <x:c r="E8"/>
+      <x:c r="F8"/>
+      <x:c r="G8"/>
+      <x:c r="H8"/>
+      <x:c r="I8"/>
+      <x:c r="J8"/>
+      <x:c r="K8"/>
+      <x:c r="L8"/>
+      <x:c r="M8"/>
+      <x:c r="N8"/>
+      <x:c r="O8"/>
+      <x:c r="P8"/>
+    </x:row>
+    <x:row r="9" ht="30" customHeight="1">
+      <x:c r="A9" s="167" t="str">
+        <x:v>Comportamento attuale</x:v>
+      </x:c>
+      <x:c r="B9" s="152" t="str">
+        <x:v>Coordina visite, trasporti e farmaci della suocera su un calendario in cucina, alternando abbreviazioni italiane e bengalesi.</x:v>
+      </x:c>
+      <x:c r="C9"/>
+      <x:c r="D9"/>
+      <x:c r="E9"/>
+      <x:c r="F9"/>
+      <x:c r="G9"/>
+      <x:c r="H9"/>
+      <x:c r="I9"/>
+      <x:c r="J9"/>
+      <x:c r="K9"/>
+      <x:c r="L9"/>
+      <x:c r="M9"/>
+      <x:c r="N9"/>
+      <x:c r="O9"/>
+      <x:c r="P9"/>
+    </x:row>
+    <x:row r="10" ht="30" customHeight="1">
+      <x:c r="A10" s="167" t="str">
+        <x:v>Esperienza con CUPweb/ER Salute</x:v>
+      </x:c>
+      <x:c r="B10" s="152" t="str">
+        <x:v>Usa bene lo smartphone nei compiti abituali; si ferma davanti a classi di priorità, primo accesso/controllo e deleghe poco chiare.</x:v>
+      </x:c>
+      <x:c r="C10"/>
+      <x:c r="D10"/>
+      <x:c r="E10"/>
+      <x:c r="F10"/>
+      <x:c r="G10"/>
+      <x:c r="H10"/>
+      <x:c r="I10"/>
+      <x:c r="J10"/>
+      <x:c r="K10"/>
+      <x:c r="L10"/>
+      <x:c r="M10"/>
+      <x:c r="N10"/>
+      <x:c r="O10"/>
+      <x:c r="P10"/>
+    </x:row>
+    <x:row r="11" ht="30" customHeight="1">
+      <x:c r="A11" s="167" t="str">
+        <x:v>Rete di aiuto</x:v>
+      </x:c>
+      <x:c r="B11" s="152" t="str">
+        <x:v>Chiede chiarimenti alla figlia, poi a medico o farmacia; conserva però il coordinamento perché conosce turni e preferenze di Nasima.</x:v>
+      </x:c>
+      <x:c r="C11"/>
+      <x:c r="D11"/>
+      <x:c r="E11"/>
+      <x:c r="F11"/>
+      <x:c r="G11"/>
+      <x:c r="H11"/>
+      <x:c r="I11"/>
+      <x:c r="J11"/>
+      <x:c r="K11"/>
+      <x:c r="L11"/>
+      <x:c r="M11"/>
+      <x:c r="N11"/>
+      <x:c r="O11"/>
+      <x:c r="P11"/>
+    </x:row>
+    <x:row r="12" ht="30" customHeight="1">
+      <x:c r="A12" s="167" t="str">
+        <x:v>Paure e frustrazioni</x:v>
+      </x:c>
+      <x:c r="B12" s="152" t="str">
+        <x:v>Teme il regime sbagliato, una duplicazione familiare o la perdita del lavoro svolto dopo un'interruzione.</x:v>
+      </x:c>
+      <x:c r="C12"/>
+      <x:c r="D12"/>
+      <x:c r="E12"/>
+      <x:c r="F12"/>
+      <x:c r="G12"/>
+      <x:c r="H12"/>
+      <x:c r="I12"/>
+      <x:c r="J12"/>
+      <x:c r="K12"/>
+      <x:c r="L12"/>
+      <x:c r="M12"/>
+      <x:c r="N12"/>
+      <x:c r="O12"/>
+      <x:c r="P12"/>
+    </x:row>
+    <x:row r="13" ht="30" customHeight="1">
+      <x:c r="A13" s="167" t="str">
+        <x:v>Condizioni di fiducia</x:v>
+      </x:c>
+      <x:c r="B13" s="152" t="str">
+        <x:v>Vuole identità e ruolo visibili, termini spiegati con esempi e uno stato finale non ambiguo da comunicare alla famiglia.</x:v>
+      </x:c>
+      <x:c r="C13"/>
+      <x:c r="D13"/>
+      <x:c r="E13"/>
+      <x:c r="F13"/>
+      <x:c r="G13"/>
+      <x:c r="H13"/>
+      <x:c r="I13"/>
+      <x:c r="J13"/>
+      <x:c r="K13"/>
+      <x:c r="L13"/>
+      <x:c r="M13"/>
+      <x:c r="N13"/>
+      <x:c r="O13"/>
+      <x:c r="P13"/>
+    </x:row>
+    <x:row r="14" ht="30" customHeight="1">
+      <x:c r="A14" s="167" t="str">
+        <x:v>Obiettivi e motivazioni</x:v>
+      </x:c>
+      <x:c r="B14" s="152" t="str">
+        <x:v>Proteggere Nasima senza dipendere sempre dalla figlia e conciliare cura, trasporti e turno di lavoro.</x:v>
+      </x:c>
+      <x:c r="C14"/>
+      <x:c r="D14"/>
+      <x:c r="E14"/>
+      <x:c r="F14"/>
+      <x:c r="G14"/>
+      <x:c r="H14"/>
+      <x:c r="I14"/>
+      <x:c r="J14"/>
+      <x:c r="K14"/>
+      <x:c r="L14"/>
+      <x:c r="M14"/>
+      <x:c r="N14"/>
+      <x:c r="O14"/>
+      <x:c r="P14"/>
+    </x:row>
+    <x:row r="15" ht="52" customHeight="1">
+      <x:c r="A15" s="167" t="str">
+        <x:v>Use case</x:v>
+      </x:c>
+      <x:c r="B15" s="152" t="str">
+        <x:v>Alle 5:50 Amina deve prenotare la fisioterapia prescritta a Nasima. Consulta impegnativa, autobus e calendario; viene interrotta e scopre che un parente potrebbe aver già telefonato. Riconosce prestazione e sede, ma esita su priorità e tipo di accesso. Deve concludere una sola prenotazione corretta e comunicarne lo stato alla famiglia.</x:v>
+      </x:c>
+      <x:c r="C15"/>
+      <x:c r="D15"/>
+      <x:c r="E15"/>
+      <x:c r="F15"/>
+      <x:c r="G15"/>
+      <x:c r="H15"/>
+      <x:c r="I15"/>
+      <x:c r="J15"/>
+      <x:c r="K15"/>
+      <x:c r="L15"/>
+      <x:c r="M15"/>
+      <x:c r="N15"/>
+      <x:c r="O15"/>
+      <x:c r="P15"/>
+    </x:row>
+    <x:row r="16" ht="52" customHeight="1">
+      <x:c r="A16" s="167"/>
+      <x:c r="B16" s="152"/>
+      <x:c r="C16"/>
+      <x:c r="D16"/>
+      <x:c r="E16"/>
+      <x:c r="F16"/>
+      <x:c r="G16"/>
+      <x:c r="H16"/>
+      <x:c r="I16"/>
+      <x:c r="J16"/>
+      <x:c r="K16"/>
+      <x:c r="L16"/>
+      <x:c r="M16"/>
+      <x:c r="N16"/>
+      <x:c r="O16"/>
+      <x:c r="P16"/>
+    </x:row>
+    <x:row r="17" ht="30" customHeight="1">
+      <x:c r="A17" s="167" t="str">
+        <x:v>Durata stimata</x:v>
+      </x:c>
+      <x:c r="B17" s="152" t="str">
+        <x:v>7-12 minuti, con possibile interruzione</x:v>
+      </x:c>
+      <x:c r="C17"/>
+      <x:c r="D17"/>
+      <x:c r="E17"/>
+      <x:c r="F17"/>
+      <x:c r="G17"/>
+      <x:c r="H17"/>
+      <x:c r="I17"/>
+      <x:c r="J17"/>
+      <x:c r="K17"/>
+      <x:c r="L17"/>
+      <x:c r="M17"/>
+      <x:c r="N17"/>
+      <x:c r="O17"/>
+      <x:c r="P17"/>
+    </x:row>
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="A18" s="167" t="str">
+        <x:v>Criterio di successo</x:v>
+      </x:c>
+      <x:c r="B18" s="152" t="str">
+        <x:v>Una sola prenotazione corretta per Nasima, compatibile con priorità, trasporto e turno; esito comprensibile e condivisibile.</x:v>
+      </x:c>
+      <x:c r="C18"/>
+      <x:c r="D18"/>
+      <x:c r="E18"/>
+      <x:c r="F18"/>
+      <x:c r="G18"/>
+      <x:c r="H18"/>
+      <x:c r="I18"/>
+      <x:c r="J18"/>
+      <x:c r="K18"/>
+      <x:c r="L18"/>
+      <x:c r="M18"/>
+      <x:c r="N18"/>
+      <x:c r="O18"/>
+      <x:c r="P18"/>
+    </x:row>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="167" t="str">
+        <x:v>Rischi osservabili</x:v>
+      </x:c>
+      <x:c r="B19" s="152" t="str">
+        <x:v>Interpretazione errata, duplicazione, perdita dei dati inseriti, abbandono verso il solo canale telefonico.</x:v>
+      </x:c>
+      <x:c r="C19"/>
+      <x:c r="D19"/>
+      <x:c r="E19"/>
+      <x:c r="F19"/>
+      <x:c r="G19"/>
+      <x:c r="H19"/>
+      <x:c r="I19"/>
+      <x:c r="J19"/>
+      <x:c r="K19"/>
+      <x:c r="L19"/>
+      <x:c r="M19"/>
+      <x:c r="N19"/>
+      <x:c r="O19"/>
+      <x:c r="P19"/>
+    </x:row>
+    <x:row r="20" ht="30" customHeight="1">
+      <x:c r="A20" s="167"/>
+      <x:c r="B20" s="152"/>
+      <x:c r="C20"/>
+      <x:c r="D20"/>
+      <x:c r="E20"/>
+      <x:c r="F20"/>
+      <x:c r="G20"/>
+      <x:c r="H20"/>
+      <x:c r="I20"/>
+      <x:c r="J20"/>
+      <x:c r="K20"/>
+      <x:c r="L20"/>
+      <x:c r="M20"/>
+      <x:c r="N20"/>
+      <x:c r="O20"/>
+      <x:c r="P20"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21"/>
+      <x:c r="B21"/>
+      <x:c r="C21"/>
+      <x:c r="D21"/>
+      <x:c r="E21" s="170" t="str">
+        <x:v>Scala diretta: 1 vicino al centro, 5 verso il bordo esterno.</x:v>
+      </x:c>
+      <x:c r="F21" s="170" t="str">
+        <x:v>Scala diretta: 1 vicino al centro, 5 verso il bordo esterno.</x:v>
+      </x:c>
+      <x:c r="G21" s="170" t="str">
+        <x:v>Scala diretta: 1 vicino al centro, 5 verso il bordo esterno.</x:v>
+      </x:c>
+      <x:c r="H21" s="170" t="str">
+        <x:v>Scala diretta: 1 vicino al centro, 5 verso il bordo esterno.</x:v>
+      </x:c>
+      <x:c r="I21" s="170" t="str">
+        <x:v>Scala diretta: 1 vicino al centro, 5 verso il bordo esterno.</x:v>
+      </x:c>
+      <x:c r="J21" s="170" t="str">
+        <x:v>Scala diretta: 1 vicino al centro, 5 verso il bordo esterno.</x:v>
+      </x:c>
+      <x:c r="K21" s="170" t="str">
+        <x:v>Scala diretta: 1 vicino al centro, 5 verso il bordo esterno.</x:v>
+      </x:c>
+      <x:c r="L21" s="170" t="str">
+        <x:v>Scala diretta: 1 vicino al centro, 5 verso il bordo esterno.</x:v>
+      </x:c>
+      <x:c r="M21" s="170" t="str">
+        <x:v>Scala diretta: 1 vicino al centro, 5 verso il bordo esterno.</x:v>
+      </x:c>
+      <x:c r="N21" s="170" t="str">
+        <x:v>Scala diretta: 1 vicino al centro, 5 verso il bordo esterno.</x:v>
+      </x:c>
+      <x:c r="O21" s="170" t="str">
+        <x:v>Scala diretta: 1 vicino al centro, 5 verso il bordo esterno.</x:v>
+      </x:c>
+      <x:c r="P21" s="170" t="str">
+        <x:v>Scala diretta: 1 vicino al centro, 5 verso il bordo esterno.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="168" t="str">
+        <x:v>Competenze e abilità</x:v>
+      </x:c>
+      <x:c r="B22" s="168" t="str">
+        <x:v>Competenze e abilità</x:v>
+      </x:c>
+      <x:c r="C22" s="168" t="str">
+        <x:v>Competenze e abilità</x:v>
+      </x:c>
+      <x:c r="D22" s="148"/>
+      <x:c r="E22" s="148"/>
+      <x:c r="F22" s="148"/>
+      <x:c r="G22" s="148"/>
+      <x:c r="H22" s="148"/>
+      <x:c r="I22"/>
+      <x:c r="J22"/>
+      <x:c r="K22"/>
+      <x:c r="L22"/>
+      <x:c r="M22"/>
+      <x:c r="N22"/>
+      <x:c r="O22"/>
+      <x:c r="P22"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="169" t="str">
+        <x:v>Dimensione</x:v>
+      </x:c>
+      <x:c r="B23" s="169" t="str">
+        <x:v>Punteggio</x:v>
+      </x:c>
+      <x:c r="C23" s="169" t="str">
+        <x:v>Motivazione</x:v>
+      </x:c>
+      <x:c r="D23" s="146"/>
+      <x:c r="E23" s="146"/>
+      <x:c r="F23" s="146"/>
+      <x:c r="G23" s="146"/>
+      <x:c r="H23" s="146"/>
+      <x:c r="I23"/>
+      <x:c r="J23"/>
+      <x:c r="K23"/>
+      <x:c r="L23"/>
+      <x:c r="M23"/>
+      <x:c r="N23"/>
+      <x:c r="O23"/>
+      <x:c r="P23"/>
+    </x:row>
+    <x:row r="24" ht="43" customHeight="1">
+      <x:c r="A24" s="152" t="str">
+        <x:v>Competenza tecnica</x:v>
+      </x:c>
+      <x:c r="B24" s="152" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C24" s="152" t="str">
+        <x:v>Usa bene lo smartphone nei compiti abituali; SPID e procedure nuove richiedono verifica.</x:v>
+      </x:c>
+      <x:c r="D24" s="152"/>
+      <x:c r="E24" s="152"/>
+      <x:c r="F24" s="152"/>
+      <x:c r="G24" s="152"/>
+      <x:c r="H24" s="152"/>
+      <x:c r="I24"/>
+      <x:c r="J24" s="166" t="str">
+        <x:v>Dimensione</x:v>
+      </x:c>
+      <x:c r="K24" s="166" t="str">
+        <x:v>Punteggio</x:v>
+      </x:c>
+      <x:c r="L24"/>
+      <x:c r="M24"/>
+      <x:c r="N24"/>
+      <x:c r="O24"/>
+      <x:c r="P24"/>
+    </x:row>
+    <x:row r="25" ht="43" customHeight="1">
+      <x:c r="A25" s="152" t="str">
+        <x:v>Competenza di dominio</x:v>
+      </x:c>
+      <x:c r="B25" s="152" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C25" s="152" t="str">
+        <x:v>Conosce routine, sedi e bisogni di Nasima, non classificazioni e deleghe amministrative.</x:v>
+      </x:c>
+      <x:c r="D25" s="152"/>
+      <x:c r="E25" s="152"/>
+      <x:c r="F25" s="152"/>
+      <x:c r="G25" s="152"/>
+      <x:c r="H25" s="152"/>
+      <x:c r="I25"/>
+      <x:c r="J25" s="166" t="str">
+        <x:v>Competenza tecnica</x:v>
+      </x:c>
+      <x:c r="K25" s="166" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L25"/>
+      <x:c r="M25"/>
+      <x:c r="N25"/>
+      <x:c r="O25"/>
+      <x:c r="P25"/>
+    </x:row>
+    <x:row r="26" ht="43" customHeight="1">
+      <x:c r="A26" s="152" t="str">
+        <x:v>Competenza linguistica</x:v>
+      </x:c>
+      <x:c r="B26" s="152" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C26" s="152" t="str">
+        <x:v>L'italiano quotidiano è funzionale; lessico sanitario scritto e sfumature burocratiche restano critici.</x:v>
+      </x:c>
+      <x:c r="D26" s="152"/>
+      <x:c r="E26" s="152"/>
+      <x:c r="F26" s="152"/>
+      <x:c r="G26" s="152"/>
+      <x:c r="H26" s="152"/>
+      <x:c r="I26"/>
+      <x:c r="J26" s="166" t="str">
+        <x:v>Competenza di dominio</x:v>
+      </x:c>
+      <x:c r="K26" s="166" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L26"/>
+      <x:c r="M26"/>
+      <x:c r="N26"/>
+      <x:c r="O26"/>
+      <x:c r="P26"/>
+    </x:row>
+    <x:row r="27" ht="43" customHeight="1">
+      <x:c r="A27" s="152" t="str">
+        <x:v>Abilità fisica e visiva</x:v>
+      </x:c>
+      <x:c r="B27" s="152" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C27" s="152" t="str">
+        <x:v>Non emergono limitazioni fisiche o visive rilevanti per il compito.</x:v>
+      </x:c>
+      <x:c r="D27" s="152"/>
+      <x:c r="E27" s="152"/>
+      <x:c r="F27" s="152"/>
+      <x:c r="G27" s="152"/>
+      <x:c r="H27" s="152"/>
+      <x:c r="I27"/>
+      <x:c r="J27" s="166" t="str">
+        <x:v>Competenza linguistica</x:v>
+      </x:c>
+      <x:c r="K27" s="166" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L27"/>
+      <x:c r="M27"/>
+      <x:c r="N27"/>
+      <x:c r="O27"/>
+      <x:c r="P27"/>
+    </x:row>
+    <x:row r="28" ht="43" customHeight="1">
+      <x:c r="A28" s="152" t="str">
+        <x:v>Motivazione</x:v>
+      </x:c>
+      <x:c r="B28" s="152" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C28" s="152" t="str">
+        <x:v>Vuole proteggere Nasima e mantenere il coordinamento familiare senza dipendere sempre dalla figlia.</x:v>
+      </x:c>
+      <x:c r="D28" s="152"/>
+      <x:c r="E28" s="152"/>
+      <x:c r="F28" s="152"/>
+      <x:c r="G28" s="152"/>
+      <x:c r="H28" s="152"/>
+      <x:c r="I28"/>
+      <x:c r="J28" s="166" t="str">
+        <x:v>Abilità fisica e visiva</x:v>
+      </x:c>
+      <x:c r="K28" s="166" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="L28"/>
+      <x:c r="M28"/>
+      <x:c r="N28"/>
+      <x:c r="O28"/>
+      <x:c r="P28"/>
+    </x:row>
+    <x:row r="29" ht="43" customHeight="1">
+      <x:c r="A29" s="152" t="str">
+        <x:v>Concentrazione</x:v>
+      </x:c>
+      <x:c r="B29" s="152" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C29" s="152" t="str">
+        <x:v>Turni, cucina condivisa, telefonate e richieste simultanee frammentano l'attenzione.</x:v>
+      </x:c>
+      <x:c r="D29" s="152"/>
+      <x:c r="E29" s="152"/>
+      <x:c r="F29" s="152"/>
+      <x:c r="G29" s="152"/>
+      <x:c r="H29" s="152"/>
+      <x:c r="I29"/>
+      <x:c r="J29" s="166" t="str">
+        <x:v>Motivazione</x:v>
+      </x:c>
+      <x:c r="K29" s="166" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="L29"/>
+      <x:c r="M29"/>
+      <x:c r="N29"/>
+      <x:c r="O29"/>
+      <x:c r="P29"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30"/>
+      <x:c r="B30"/>
+      <x:c r="C30"/>
+      <x:c r="D30"/>
+      <x:c r="E30"/>
+      <x:c r="F30"/>
+      <x:c r="G30"/>
+      <x:c r="H30"/>
+      <x:c r="I30"/>
+      <x:c r="J30" s="166" t="str">
+        <x:v>Concentrazione</x:v>
+      </x:c>
+      <x:c r="K30" s="166" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L30"/>
+      <x:c r="M30"/>
+      <x:c r="N30"/>
+      <x:c r="O30"/>
+      <x:c r="P30"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A2:P2"/>
+    <x:mergeCell ref="A22:C22"/>
+    <x:mergeCell ref="E21:P21"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3e895a39d1e4773"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: update Phase B personas with detailed profiles and scenarios
</commit_message>
<xml_diff>
--- a/phase-b/phase-b-personas-and-cast.xlsx
+++ b/phase-b/phase-b-personas-and-cast.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="1" r:id="Rb9dc9098233a4371"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cast" sheetId="2" r:id="R62c6d0de86db4895"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence map" sheetId="3" r:id="R82adbb1f644247f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario #1" sheetId="4" r:id="R231400425f4f45ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario #2" sheetId="5" r:id="Ra0a0a8b59c014a4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario #3" sheetId="6" r:id="R8f684165dc774d70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario #4" sheetId="7" r:id="R619b238ad69f4e72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="1" r:id="R61da85e44b084011"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cast" sheetId="2" r:id="R7ede86045a964a6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence map" sheetId="3" r:id="R2101c85db1b64e89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario #1" sheetId="4" r:id="R5e7475075a204832"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario #2" sheetId="5" r:id="R23a7264b078c403f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario #3" sheetId="6" r:id="Rdda1600592664ac8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario #4" sheetId="7" r:id="R355ee3bf9de4470a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1777,7 +1777,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R40c4fdaff3e64c2d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R016c893124b64c5c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1812,7 +1812,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R084733f41045491e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R667a0292712241db"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1847,7 +1847,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R26cfc401e78b43a2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1847aebf38114e1b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1882,7 +1882,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1d357e1fec254fc2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Red720e21d0124256"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1917,7 +1917,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rca0b1e57448d446a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0cf330eef383408c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -4780,7 +4780,7 @@
     <x:mergeCell ref="A42:D42"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2eda4a0203e44c36"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46afa7aa59e14488"/>
 </x:worksheet>
 </file>
 
@@ -6348,7 +6348,7 @@
         <x:v>Citazione provvisoria</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str">
-        <x:v>Se non c'è qualcuno che mi aiuta, io non riesco a prenotare niente da sola.</x:v>
+        <x:v>Le date le segno sul calendario vicino al telefono; sullo schermo ho paura di premere la cosa sbagliata.</x:v>
       </x:c>
       <x:c r="C9" s="2"/>
       <x:c r="D9" s="2"/>
@@ -6370,7 +6370,7 @@
         <x:v>Comportamento attuale</x:v>
       </x:c>
       <x:c r="B10" s="16" t="str">
-        <x:v>Preferisce farmacia e telefono; prova l'app solo quando la figlia non è disponibile.</x:v>
+        <x:v>Conserva impegnative e ricevute in una busta blu nel cassetto del telefono; incrocia i documenti con calendario cartaceo e orari dell'autobus.</x:v>
       </x:c>
       <x:c r="C10" s="2"/>
       <x:c r="D10" s="2"/>
@@ -6392,7 +6392,7 @@
         <x:v>Esperienza con CUPweb/ER Salute</x:v>
       </x:c>
       <x:c r="B11" s="16" t="str">
-        <x:v>Ha tentato ER Salute, ma autenticazione, etichette poco evidenti e messaggi di errore l'hanno portata ad abbandonare.</x:v>
+        <x:v>Ha provato ER Salute, ma SPID, azioni testuali e messaggi di errore poco comprensibili l'hanno portata ad abbandonare.</x:v>
       </x:c>
       <x:c r="C11" s="2"/>
       <x:c r="D11" s="2"/>
@@ -6414,7 +6414,7 @@
         <x:v>Rete di aiuto</x:v>
       </x:c>
       <x:c r="B12" s="16" t="str">
-        <x:v>Chiama Elena, che vive a distanza e spesso completa la pratica al posto suo.</x:v>
+        <x:v>Elena interviene quando Pina non riconosce il passo successivo o teme una conseguenza irreversibile, non per ogni scelta.</x:v>
       </x:c>
       <x:c r="C12" s="2"/>
       <x:c r="D12" s="2"/>
@@ -6436,7 +6436,7 @@
         <x:v>Paure e frustrazioni</x:v>
       </x:c>
       <x:c r="B13" s="16" t="str">
-        <x:v>Teme di sbagliare, perdere una prenotazione, pagare per errore o non riuscire a recuperare.</x:v>
+        <x:v>Teme di premere l'azione sbagliata, perdere la prenotazione o non riuscire a recuperare dopo un errore.</x:v>
       </x:c>
       <x:c r="C13" s="2"/>
       <x:c r="D13" s="2"/>
@@ -6458,7 +6458,7 @@
         <x:v>Condizioni di fiducia</x:v>
       </x:c>
       <x:c r="B14" s="16" t="str">
-        <x:v>Passaggi brevi, linguaggio rassicurante, conferme esplicite e un aiuto raggiungibile senza ricominciare.</x:v>
+        <x:v>Si fida di azioni grandi, linguaggio quotidiano, conferme chiare e possibilità di recupero.</x:v>
       </x:c>
       <x:c r="C14" s="2"/>
       <x:c r="D14" s="2"/>
@@ -6480,7 +6480,7 @@
         <x:v>Obiettivi e motivazioni</x:v>
       </x:c>
       <x:c r="B15" s="16" t="str">
-        <x:v>Completare in autonomia almeno le prenotazioni ricorrenti e sentirsi ancora indipendente.</x:v>
+        <x:v>Mantenere l'indipendenza e scegliere appuntamenti raggiungibili in autobus dopo le 10, senza sentirsi giudicata.</x:v>
       </x:c>
       <x:c r="C15" s="2"/>
       <x:c r="D15" s="2"/>
@@ -6502,7 +6502,7 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="B16" s="16" t="str">
-        <x:v>Pina, 78 anni, deve prenotare la visita diabetologica di controllo semestrale. Apre ER Salute sul proprio smartphone, ma non ricorda come completare l'accesso e non distingue subito l'azione per prenotare dalle informazioni generali. Dopo due tentativi e un messaggio che non comprende, chiama Elena durante una riunione. Pina vorrebbe proseguire personalmente, ma finisce per lasciare alla figlia l'intera pratica.</x:v>
+        <x:v>Pina recupera l'impegnativa dalla busta blu, evita il mercato del martedì e verifica l'autobus. Poi prova ER Salute: non ricorda la password SPID, confonde Prenota con Informazioni e non comprende un errore. Dopo due tentativi chiama Elena. Deve scegliere sede e data consapevolmente e ricevere una conferma verificabile senza essere sostituita.</x:v>
       </x:c>
       <x:c r="C16" s="2"/>
       <x:c r="D16" s="2"/>
@@ -7430,7 +7430,7 @@
     <x:mergeCell ref="E21:P21"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1e06d1348d548d1"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2f30b77ad624b3b"/>
 </x:worksheet>
 </file>
 
@@ -7656,7 +7656,7 @@
         <x:v>Citazione provvisoria</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str">
-        <x:v>Vorrei che mia madre potesse cavarsela da sola per le cose semplici, così mi preoccuperei solo per l'importante.</x:v>
+        <x:v>Se la guido al telefono per dieci minuti, poi non so se l'ho aiutata o se ho fatto tutto io.</x:v>
       </x:c>
       <x:c r="C9" s="2"/>
       <x:c r="D9" s="2"/>
@@ -7678,7 +7678,7 @@
         <x:v>Comportamento attuale</x:v>
       </x:c>
       <x:c r="B10" s="16" t="str">
-        <x:v>Gestisce da remoto prenotazioni e disdette della madre, spesso durante pause lavorative.</x:v>
+        <x:v>Segna gli appuntamenti di Pina in rosso sul calendario digitale e conserva numeri e domande in una nota protetta; rifiuta password inviate in chat.</x:v>
       </x:c>
       <x:c r="C10" s="2"/>
       <x:c r="D10" s="2"/>
@@ -7700,7 +7700,7 @@
         <x:v>Esperienza con CUPweb/ER Salute</x:v>
       </x:c>
       <x:c r="B11" s="16" t="str">
-        <x:v>Usa senza difficoltà SPID e servizi digitali, ma trova oneroso ricostruire ogni volta contesto e stato delle pratiche della madre.</x:v>
+        <x:v>Conosce CUPweb ed ER Salute, ma deve ricostruire dati, credenziali e intenzione della madre a ogni richiesta.</x:v>
       </x:c>
       <x:c r="C11" s="2"/>
       <x:c r="D11" s="2"/>
@@ -7722,7 +7722,7 @@
         <x:v>Rete di aiuto</x:v>
       </x:c>
       <x:c r="B12" s="16" t="str">
-        <x:v>È il principale punto di riferimento di Pina e tende a prendere il controllo quando il tempo è poco.</x:v>
+        <x:v>È il riferimento a distanza di Pina; interviene nei casi complessi e cerca di non assumere il controllo delle azioni semplici.</x:v>
       </x:c>
       <x:c r="C12" s="2"/>
       <x:c r="D12" s="2"/>
@@ -7744,7 +7744,7 @@
         <x:v>Paure e frustrazioni</x:v>
       </x:c>
       <x:c r="B13" s="16" t="str">
-        <x:v>Teme no-show, scadenze perse e azioni duplicate; teme anche che Pina rinunci del tutto a imparare.</x:v>
+        <x:v>Teme errori sul profilo sbagliato, notifiche insufficienti e che l'efficienza trasformi l'aiuto in controllo permanente.</x:v>
       </x:c>
       <x:c r="C13" s="2"/>
       <x:c r="D13" s="2"/>
@@ -7766,7 +7766,7 @@
         <x:v>Condizioni di fiducia</x:v>
       </x:c>
       <x:c r="B14" s="16" t="str">
-        <x:v>Vuole visibilità sullo stato, notifiche comprensibili e confini chiari tra assistenza, delega e conferma finale.</x:v>
+        <x:v>Accetta la delega se identità, conseguenze e informazione a Pina restano esplicite; non vuole scambi informali di credenziali.</x:v>
       </x:c>
       <x:c r="C14" s="2"/>
       <x:c r="D14" s="2"/>
@@ -7788,7 +7788,7 @@
         <x:v>Obiettivi e motivazioni</x:v>
       </x:c>
       <x:c r="B15" s="16" t="str">
-        <x:v>Ridurre le interruzioni e trasformarsi da esecutrice a guida, senza perdere il controllo sulle situazioni critiche.</x:v>
+        <x:v>Ridurre le emergenze e le interruzioni, lasciando a Pina le decisioni semplici e mantenendo il proprio intervento per i casi complessi.</x:v>
       </x:c>
       <x:c r="C15" s="2"/>
       <x:c r="D15" s="2"/>
@@ -7810,7 +7810,7 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="B16" s="16" t="str">
-        <x:v>Durante una riunione Elena riceve una chiamata da Pina, che non riesce a disdire una visita dopo un cambio di programma. Elena apre l'app da remoto, individua la prenotazione corretta e risolve la pratica in pochi minuti. Anche questa volta l'urgenza la spinge a sostituirsi alla madre, sebbene desideri che Pina impari a gestire almeno le azioni a basso rischio.</x:v>
+        <x:v>Durante la chiusura mensile delle paghe Elena riceve una chiamata da Pina: una visita va disdetta. Ha una riunione tra cinque minuti e una collega attende risposta. Deve identificare profilo e appuntamento, controllare le conseguenze e rassicurare la madre senza chiederle credenziali in chat. Il risultato deve essere verificabile da entrambe.</x:v>
       </x:c>
       <x:c r="C16" s="2"/>
       <x:c r="D16" s="2"/>
@@ -8738,7 +8738,7 @@
     <x:mergeCell ref="E21:P21"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf9974b9f3a54863"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13122d37ed48459c"/>
 </x:worksheet>
 </file>
 
@@ -8964,7 +8964,7 @@
         <x:v>Citazione provvisoria</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str">
-        <x:v>Se capisco cosa sto confermando, preferisco fare da solo e chiedere aiuto solo quando serve.</x:v>
+        <x:v>Non mi serve che mi dicano che è facile: mi serve capire costo e conseguenze prima di confermare.</x:v>
       </x:c>
       <x:c r="C9" s="2"/>
       <x:c r="D9" s="2"/>
@@ -8986,7 +8986,7 @@
         <x:v>Comportamento attuale</x:v>
       </x:c>
       <x:c r="B10" s="16" t="str">
-        <x:v>Prenota spesso in farmacia o al telefono, ma usa i servizi online quando il percorso gli appare prevedibile.</x:v>
+        <x:v>Usa il tablet al tavolo della cucina, annota i passaggi nuovi su un quaderno e salva o stampa le conferme per la bacheca condivisa con Paola.</x:v>
       </x:c>
       <x:c r="C10" s="2"/>
       <x:c r="D10" s="2"/>
@@ -9008,7 +9008,7 @@
         <x:v>Esperienza con CUPweb/ER Salute</x:v>
       </x:c>
       <x:c r="B11" s="16" t="str">
-        <x:v>Ha già usato SPID e il Fascicolo Sanitario; abbandona quando incontra etichette burocratiche, controlli piccoli o differenze non spiegate tra SSN e libera professione.</x:v>
+        <x:v>Usa SPID e servizi digitali; si ferma davanti a SSN, libera professione e costi o conseguenze non immediatamente visibili.</x:v>
       </x:c>
       <x:c r="C11" s="2"/>
       <x:c r="D11" s="2"/>
@@ -9030,7 +9030,7 @@
         <x:v>Rete di aiuto</x:v>
       </x:c>
       <x:c r="B12" s="16" t="str">
-        <x:v>Chiede al figlio una conferma puntuale, non vuole che completi l'intera procedura al posto suo.</x:v>
+        <x:v>Chiede al figlio una verifica puntuale, non l'esecuzione completa; condivide calendario e conferme con la moglie Paola.</x:v>
       </x:c>
       <x:c r="C12" s="2"/>
       <x:c r="D12" s="2"/>
@@ -9052,7 +9052,7 @@
         <x:v>Paure e frustrazioni</x:v>
       </x:c>
       <x:c r="B13" s="16" t="str">
-        <x:v>Teme di scegliere il regime errato, accettare un costo non previsto o perdere quanto già inserito tornando indietro.</x:v>
+        <x:v>Teme una conferma onerosa, una sede sbagliata o di perdere le scelte tornando indietro.</x:v>
       </x:c>
       <x:c r="C13" s="2"/>
       <x:c r="D13" s="2"/>
@@ -9074,7 +9074,7 @@
         <x:v>Condizioni di fiducia</x:v>
       </x:c>
       <x:c r="B14" s="16" t="str">
-        <x:v>Vuole vedere costi, conseguenze e stato della pratica prima della conferma, con la possibilità di correggere senza ricominciare.</x:v>
+        <x:v>Vuole leggere con calma, correggere senza ricominciare e archiviare una conferma leggibile; rifiuta toni paternalistici.</x:v>
       </x:c>
       <x:c r="C14" s="2"/>
       <x:c r="D14" s="2"/>
@@ -9096,7 +9096,7 @@
         <x:v>Obiettivi e motivazioni</x:v>
       </x:c>
       <x:c r="B15" s="16" t="str">
-        <x:v>Gestire autonomamente le prenotazioni ordinarie con un percorso rapido, senza spiegazioni paternalistiche.</x:v>
+        <x:v>Gestire autonomamente le prenotazioni ordinarie, mantenendo il figlio come verifica mirata e non come sostituto.</x:v>
       </x:c>
       <x:c r="C15" s="2"/>
       <x:c r="D15" s="2"/>
@@ -9118,7 +9118,7 @@
         <x:v>Use case</x:v>
       </x:c>
       <x:c r="B16" s="16" t="str">
-        <x:v>Renato, 70 anni, riceve la prescrizione per un controllo oculistico annuale. A casa usa il tablet e accede con SPID. Trova la prestazione, ma si ferma quando deve distinguere tra Servizio Sanitario Nazionale e libera professione e quando l'elenco delle disponibilità richiede selezioni precise. Chiama il figlio per una conferma sul significato delle opzioni, poi vuole proseguire e controllare personalmente costo, sede e data prima della conferma.</x:v>
+        <x:v>Dopo colazione Renato confronta due sedi dal tablet, consulta il calendario condiviso con Paola e evita il turno all'archivio storico. Si ferma sulla distinzione tra SSN e libera professione. Deve comprenderne costo e conseguenze, mantenere le scelte e archiviare una conferma leggibile senza cedere il compito al figlio.</x:v>
       </x:c>
       <x:c r="C16" s="2"/>
       <x:c r="D16" s="2"/>
@@ -10046,7 +10046,7 @@
     <x:mergeCell ref="E21:P21"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra828350eeb6e430c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb86e98ccab641d8"/>
 </x:worksheet>
 </file>
 
@@ -10781,6 +10781,6 @@
     <x:mergeCell ref="E21:P21"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3e895a39d1e4773"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37ea69367d084964"/>
 </x:worksheet>
 </file>
</xml_diff>